<commit_message>
Batch 2 one file not updated issue fix-1
</commit_message>
<xml_diff>
--- a/Master-sheet/07-Test-Master-File.xlsx
+++ b/Master-sheet/07-Test-Master-File.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19155" windowHeight="6345"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19152" windowHeight="6348"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
     <t>\\192.168.1.237\Accounts\SURESH_KAKEE_AUTOMATION PROJECTS\PRODUCTION AND DISPATCH\05. UDYAMNAGAR\07. MANOJ KANDHARE\Quantity Report - UN-RM.xlsb</t>
   </si>
   <si>
-    <t>\\192.168.1.237\Accounts\SURESH_KAKEE_AUTOMATION PROJECTS\MARKETING EMPLOYEES\001 Production\01 2025-26\002 UDYAMNAGAR\UDYAM-SH &amp; RF Stock Report.xlsb</t>
+    <t>\\192.168.1.237\Accounts\SURESH_KAKEE_AUTOMATION PROJECTS\SOLAPUR (HO)\04. MARKETING\A. IRRIGATION DIVISION\10. GANGADHAR PARDHE\Sales Quantity Base Report - 2025-26_New_17-11-25.xlsb</t>
   </si>
 </sst>
 </file>
@@ -396,15 +396,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="44" customWidth="1"/>
-    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -420,7 +420,7 @@
       </c>
       <c r="F1" s="2"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -431,7 +431,7 @@
         <v>0.625</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -447,8 +447,8 @@
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B3" r:id="rId1"/>
-    <hyperlink ref="B2" r:id="rId2"/>
+    <hyperlink ref="B2" r:id="rId1"/>
+    <hyperlink ref="B3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>